<commit_message>
work progress after design changes
</commit_message>
<xml_diff>
--- a/documentation/metadata.xlsx
+++ b/documentation/metadata.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repo\Sloth\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B6F9E49-7F82-46C8-8168-AA67BA6AFC8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C86174-1954-4A22-AE8C-3497E17A0F04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="link" sheetId="1" r:id="rId1"/>
-    <sheet name="nav-panel" sheetId="2" r:id="rId2"/>
+    <sheet name="side-panel" sheetId="2" r:id="rId2"/>
+    <sheet name="header-panel" sheetId="3" r:id="rId3"/>
+    <sheet name="nav-panel" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>icon</t>
   </si>
@@ -38,12 +40,6 @@
   </si>
   <si>
     <t>warningCount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type </t>
-  </si>
-  <si>
-    <t>side-nav, header-nav, drop-down-nav</t>
   </si>
 </sst>
 </file>
@@ -391,18 +387,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D44DC8F3-3705-4B00-8FBD-9AC18FDFC56C}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF8AA2A7-AB94-491B-BC98-E06211493A03}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C94CF39D-1EC3-4390-8291-276EEDB6F255}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>